<commit_message>
Update Victoria University partnership proposal deck script and associated PowerPoint presentation. Adjusted branding details for clarity, improved layout dimensions, and refined text formatting. Updated images in the presentation to align with the latest assets.
</commit_message>
<xml_diff>
--- a/opportunities/tracker.xlsx
+++ b/opportunities/tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\coding\apps\flutter\fairbanks\opportunities\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0A6DA81-3109-4107-A11A-1D8BAEE1207C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A116C12-FFE1-4627-9083-7A8933925C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Scan Notes" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Opportunities!$A$1:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Opportunities!$A$1:$I$6</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="82">
   <si>
     <t>Project Title</t>
   </si>
@@ -111,21 +111,6 @@
   </si>
   <si>
     <t>unknown</t>
-  </si>
-  <si>
-    <t>DPI Safeguards Accelerator (UN ODET / UNDP)</t>
-  </si>
-  <si>
-    <t>https://www.dpi-safeguards.org/accelerator</t>
-  </si>
-  <si>
-    <t>Cohort programme helping partners embed practical safeguards into active Digital Public Infrastructure. NGO pathway for Uganda: issue-specific work on FairBanks FCHIP (consent/data use, offline inclusion, grievance). Catalytic grant up to USD 70,000 over 6-9 months, plus tools and peer learning. Stage 1 Airtable screening; Stage 2 needs government letter if longlisted. FairBanks submitted as community-based health operator with live FCHIP MVP.</t>
-  </si>
-  <si>
-    <t>30 July 2026</t>
-  </si>
-  <si>
-    <t>applications/dpi-safeguards</t>
   </si>
   <si>
     <t>U.S. Dept of State — Uganda Health System MOU (up to $60M)</t>
@@ -423,7 +408,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -481,9 +466,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -826,7 +808,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="3" width="42.1796875" customWidth="1"/>
@@ -951,90 +933,90 @@
       </c>
       <c r="I4" s="4"/>
     </row>
-    <row r="5" spans="1:9" ht="169.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:9" ht="156.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H6" s="15">
+        <v>46225</v>
+      </c>
+      <c r="I6" s="4"/>
+    </row>
+    <row r="7" spans="1:9" ht="117" x14ac:dyDescent="0.35">
+      <c r="A7" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="14">
-        <v>46232</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" ht="156.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" s="4" t="s">
+      <c r="H7" s="19">
+        <v>46225</v>
+      </c>
+      <c r="I7" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="15">
-        <v>46225</v>
-      </c>
-      <c r="I7" s="4"/>
-    </row>
-    <row r="8" spans="1:9" ht="110" customHeight="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="8" spans="1:9" ht="117" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
         <v>44</v>
       </c>
@@ -1045,7 +1027,7 @@
         <v>46</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E8" s="18" t="s">
         <v>20</v>
@@ -1060,38 +1042,10 @@
         <v>46225</v>
       </c>
       <c r="I8" s="16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="G9" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="19">
-        <v>46225</v>
-      </c>
-      <c r="I9" s="16" t="s">
-        <v>52</v>
-      </c>
-    </row>
+    </row>
+    <row r="9" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="11" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="12" spans="1:9" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1104,16 +1058,14 @@
     <row r="19" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="20" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
     <row r="21" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="22" ht="92.25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
-  <autoFilter ref="A1:I7" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:I6" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
     <hyperlink ref="B4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="B5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="B6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="B7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="B6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -1132,138 +1084,138 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="65" x14ac:dyDescent="0.35">
       <c r="A16" s="20" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B16" s="20" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add initial files for CDC-RFA-JG-26-0056 FairBanks grant application, including project narrative, compliance documents, and source of truth guidelines. These files support the submission process and ensure alignment with Grants.gov requirements.
</commit_message>
<xml_diff>
--- a/opportunities/tracker.xlsx
+++ b/opportunities/tracker.xlsx
@@ -18,10 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -109,7 +108,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -147,12 +146,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -218,7 +231,13 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -624,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="42.1796875" customWidth="1" min="1" max="3"/>
@@ -892,7 +911,7 @@
           <t>Submitted</t>
         </is>
       </c>
-      <c r="H6" s="23" t="n">
+      <c r="H6" s="24" t="n">
         <v>46243</v>
       </c>
       <c r="I6" s="16" t="inlineStr">
@@ -1032,7 +1051,49 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="92.25" customHeight="1"/>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>CDC - Strengthening Global Health Security detect/notify/respond globally (CDC-RFA-JG-26-0056)</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="inlineStr">
+        <is>
+          <t>https://simpler.grants.gov/opportunity/8454e463-cd43-4d0d-97a2-8a4310e0ce6b</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>CDC cooperative agreement (93.318) to strengthen country capacity to detect, notify, and respond to outbreaks globally via MoH partnerships. Year 1 pool about USD 24M; 4-8 awards; Component 1 ceiling USD 3M. For-profit and foreign entities eligible; Uganda local partner +10 points. FairBanks Year 1 Uganda-primary with FCHIP last-mile surveillance under MoH. Confirm multi-country LOIs and SAM/UEI before submit. Deadline 14 August 2026.</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>14 August 2026 (11:59 p.m. ET)</t>
+        </is>
+      </c>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>Multi-gender (all genders)</t>
+        </is>
+      </c>
+      <c r="F10" s="25" t="inlineStr">
+        <is>
+          <t>Drafting</t>
+        </is>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="inlineStr"/>
+      <c r="I10" s="25" t="inlineStr">
+        <is>
+          <t>applications/cdc-ghs-global</t>
+        </is>
+      </c>
+    </row>
     <row r="11" ht="92.25" customHeight="1"/>
     <row r="12" ht="92.25" customHeight="1"/>
     <row r="13" ht="92.25" customHeight="1"/>

</xml_diff>